<commit_message>
Run: Updated Rohin job outputs 2026-06-04 16:12:58
</commit_message>
<xml_diff>
--- a/users/Rohin/outputs/JobMatches.xlsx
+++ b/users/Rohin/outputs/JobMatches.xlsx
@@ -10,6 +10,7 @@
     <sheet name="20260604_1046" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="20260604_1157" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="20260604_134415" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="20260604_161235" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1563,15 +1564,734 @@
           <t>2026-06-04</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Grob Aircraft</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Offene Stellen - Grob Aircraft SE</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://jobs.grob-aircraft.com/jobs</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>85</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation, Design</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Fraunhofer</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Wissenschaftliche/r Mitarbeiter/in FPGA-Entwicklung und Regelungstechnik (all genders) Stellendetails | Fraunhofer-Gesellschaft</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://jobs.fraunhofer.de/job/Dresden-Wissenschaftlicher-Mitarbeiterin-FPGA-Entwicklung-und-Regelungstechnik-%28all-genders%29-01109/1381190933/</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>85</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation, Design</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>AIP Services</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Jobs: Entwicklungsingenieur Leistungselektronik (m/w/d) in Altenstadt | Aviation Industry Personnel SERVICES GmbH</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://k21840.coveto.de/job-entwicklungsingenieur-leistungselektronik-m-w-d-altenstadt-14261.html</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>85</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation, Design</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Fraunhofer</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Fraunhofer-Gesellschaft Jobs</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://jobs.fraunhofer.de/search/</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>85</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation, Design</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Rocket Factory</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Bewerbung als Einkäufer (m/f/d) bei Rocket Factory Augsburg AG</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/rocketfactoryaugsburgag/jobs/4845549101</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>50</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Entwicklung, Design</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Germany, UK</t>
+        </is>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ÒKAPI</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Team Lead Java Development (m/w/d) | Jobs bei OKAPI:Orbits GmbH</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://okapiorbits.jobs.personio.de/job/2573721</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>45</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Entwicklung</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Germany, UK</t>
+        </is>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Grob Aircraft</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Electrical Designer / ECAD Administrator (m/f/d) – Siemens Capital Harness | Aerospace - Grob Aircraft SE</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://jobs.grob-aircraft.com/jobs/7608802-electrical-designer-ecad-administrator-m-f-d-siemens-capital-harness-aerospace</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>45</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Entwicklung, Design</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Grob Aircraft</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Avionics / Electrical Designer (m/f/d) - Grob Aircraft SE</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://jobs.grob-aircraft.com/jobs/7601670-avionics-electrical-designer-m-f-d</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>40</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Entwicklung, Design</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>volkswagen</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Volkswagen Group Services Gmbh | Job Portal</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://jobs.volkswagen-group.com/Volkswagen-Group-Services/?locale=de_DE</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>40</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Entwicklung, Design</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L10" t="b">
+        <v>1</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ENERCON</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Technology Project Manager (m/f/d) Job Details | ENERCON</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://career.enercon.de/job/Aurich-Technology-Project-Manager-%28mfd%29-NI-26605/1353733755/</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>40</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Entwicklung, Design</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L11" t="b">
+        <v>1</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Fraunhofer</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Stud. Hilfskraft (m/w/d): Design/Konzeption &amp; Umsetzung einer Robotik-Zelle für Laborautomatisierung Stellendetails | Fraunhofer-Gesellschaft</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://jobs.fraunhofer.de/job/Stuttgart-Stud_-Hilfskraft-%28mwd%29-DesignKonzeption-&amp;-Umsetzung-einer-Robotik-Zelle-f%C3%BCr-Laborautomatisierung-70569/1390751233/</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>40</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Entwicklung, Design</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L12" t="b">
+        <v>1</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>CrawlDate</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>PostedDate</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Keywords</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Locations</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Grob Aircraft</t>
+          <t>PhysicsX</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>England</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1581,20 +2301,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Offene Stellen - Grob Aircraft SE</t>
+          <t>Job Application for Senior Simulation Data Engineer at PhysicsX</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://jobs.grob-aircraft.com/jobs</t>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4789254101</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>85</v>
+        <v>225</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Entwicklung, Simulation, Design</t>
+          <t>CFD, Simulation, OpenFOAM, Simulation Engineer, StarCCM, ANSYS, Design</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -1625,12 +2345,12 @@
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Fraunhofer</t>
+          <t>PhysicsX</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>England</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1640,20 +2360,20 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Wissenschaftliche/r Mitarbeiter/in FPGA-Entwicklung und Regelungstechnik (all genders) Stellendetails | Fraunhofer-Gesellschaft</t>
+          <t>Job Application for Principal CFD Engineer at PhysicsX</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://jobs.fraunhofer.de/job/Dresden-Wissenschaftlicher-Mitarbeiterin-FPGA-Entwicklung-und-Regelungstechnik-%28all-genders%29-01109/1381190933/</t>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4763024101</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>85</v>
+        <v>210</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Entwicklung, Simulation, Design</t>
+          <t>CFD, Simulation, Fluid, OpenFOAM, Simulation Engineer, Design</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -1684,12 +2404,12 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>AIP Services</t>
+          <t>PhysicsX</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>England</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1699,20 +2419,20 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Jobs: Entwicklungsingenieur Leistungselektronik (m/w/d) in Altenstadt | Aviation Industry Personnel SERVICES GmbH</t>
+          <t>Job Application for Senior CFD Engineer at PhysicsX</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://k21840.coveto.de/job-entwicklungsingenieur-leistungselektronik-m-w-d-altenstadt-14261.html</t>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4750020101</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>85</v>
+        <v>195</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Entwicklung, Simulation, Design</t>
+          <t>CFD, Simulation, Fluid, OpenFOAM, Design</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1743,12 +2463,12 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Fraunhofer</t>
+          <t>PhysicsX</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>England</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1758,20 +2478,20 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Fraunhofer-Gesellschaft Jobs</t>
+          <t>Job Application for Senior CFD Engineer - Multiphase at PhysicsX</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://jobs.fraunhofer.de/search/</t>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4845687101</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>85</v>
+        <v>195</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Entwicklung, Simulation, Design</t>
+          <t>CFD, Simulation, Fluid, OpenFOAM, Design</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1802,12 +2522,12 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Rocket Factory</t>
+          <t>PhysicsX</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>England</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1817,25 +2537,25 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Bewerbung als Einkäufer (m/f/d) bei Rocket Factory Augsburg AG</t>
+          <t>Job Application for Senior CFD Engineer - Turbomachinery at PhysicsX</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/rocketfactoryaugsburgag/jobs/4845549101</t>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4644845101</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>50</v>
+        <v>145</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Entwicklung, Design</t>
+          <t>CFD, Simulation, Fluid, ANSYS, Design</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Germany, UK</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="L6" t="b">
@@ -1861,12 +2581,12 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ÒKAPI</t>
+          <t>PhysicsX</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>England</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1876,25 +2596,25 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Team Lead Java Development (m/w/d) | Jobs bei OKAPI:Orbits GmbH</t>
+          <t>Job Application for Principal Machine Learning Engineer at PhysicsX</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://okapiorbits.jobs.personio.de/job/2573721</t>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4749999101</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>45</v>
+        <v>100</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Entwicklung</t>
+          <t>CFD, Simulation, Simulation Engineer, Design</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Germany, UK</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="L7" t="b">
@@ -1920,12 +2640,12 @@
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Grob Aircraft</t>
+          <t>PhysicsX</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>England</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1935,25 +2655,25 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Electrical Designer / ECAD Administrator (m/f/d) – Siemens Capital Harness | Aerospace - Grob Aircraft SE</t>
+          <t>Job Application for Machine Learning Engineer at PhysicsX</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://jobs.grob-aircraft.com/jobs/7608802-electrical-designer-ecad-administrator-m-f-d-siemens-capital-harness-aerospace</t>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4749996101</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>45</v>
+        <v>100</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Entwicklung, Design</t>
+          <t>CFD, Simulation, Simulation Engineer, Design</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="L8" t="b">
@@ -1979,12 +2699,12 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Grob Aircraft</t>
+          <t>PhysicsX</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>England</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1994,20 +2714,20 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Avionics / Electrical Designer (m/f/d) - Grob Aircraft SE</t>
+          <t>Job Application for Principal Machine Learning Infrastructure Engineer at PhysicsX</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://jobs.grob-aircraft.com/jobs/7601670-avionics-electrical-designer-m-f-d</t>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4789202101</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Entwicklung, Design</t>
+          <t>CFD, Simulation, Simulation Engineer, Design</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -2038,12 +2758,12 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>volkswagen</t>
+          <t>PhysicsX</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>England</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -2053,20 +2773,20 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Volkswagen Group Services Gmbh | Job Portal</t>
+          <t>Job Application for Senior Machine Learning Engineer at PhysicsX</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://jobs.volkswagen-group.com/Volkswagen-Group-Services/?locale=de_DE</t>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4678291101</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Entwicklung, Design</t>
+          <t>CFD, Simulation, Simulation Engineer, Design</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -2097,12 +2817,12 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ENERCON</t>
+          <t>PhysicsX</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>England</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -2112,20 +2832,20 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Technology Project Manager (m/f/d) Job Details | ENERCON</t>
+          <t>Job Application for Senior FEA Engineer at PhysicsX</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://career.enercon.de/job/Aurich-Technology-Project-Manager-%28mfd%29-NI-26605/1353733755/</t>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4750023101</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Entwicklung, Design</t>
+          <t>Simulation, Fluid, ANSYS, Design</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -2156,46 +2876,1462 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Fraunhofer</t>
+          <t>PhysicsX</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Job Application for Simulation Engineer - FEA at PhysicsX</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4845916101</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>85</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Simulation, Simulation Engineer, ANSYS, Design</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L12" t="b">
+        <v>1</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>PhysicsX</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Job Application for Senior Simulation Engineer - Electromagnetics Specialist at PhysicsX</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4871700101</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>85</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Simulation, Simulation Engineer, ANSYS, Design</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L13" t="b">
+        <v>1</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Mbda</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Job</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Stud. Hilfskraft (m/w/d): Design/Konzeption &amp; Umsetzung einer Robotik-Zelle für Laborautomatisierung Stellendetails | Fraunhofer-Gesellschaft</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>https://jobs.fraunhofer.de/job/Stuttgart-Stud_-Hilfskraft-%28mwd%29-DesignKonzeption-&amp;-Umsetzung-einer-Robotik-Zelle-f%C3%BCr-Laborautomatisierung-70569/1390751233/</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Datenschutz – Karriereportal MBDA Deutschland</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://www.mbda-careers.de/datenschutz/</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>85</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Entwicklung, FSI, Design</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L14" t="b">
+        <v>1</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Mbda</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Standorte – Karriereportal MBDA Deutschland</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://www.mbda-careers.de/arbeitgeber/standorte/</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>80</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L15" t="b">
+        <v>1</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>PhysicsX</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Job Application for Senior Computer Vision Data Scientist at PhysicsX</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4852973101</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>80</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Simulation, Fluid, Design</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L16" t="b">
+        <v>1</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Mbda</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>MBDA Deutschland – Karriereportal MBDA Deutschland</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.mbda-careers.de/arbeitgeber/unternehmen/mbda-deutschland/</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>80</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L17" t="b">
+        <v>1</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Mbda</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Schrobenhausen – Karriereportal MBDA Deutschland</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://www.mbda-careers.de/arbeitgeber/standorte/schrobenhausen/</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>80</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L18" t="b">
+        <v>1</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>PhysicsX</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Job Application for Research Scientist at PhysicsX</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4652632101</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>75</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Simulation, Simulation Engineer, Design</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L19" t="b">
+        <v>1</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>PhysicsX</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Job Application for Principal Research Scientist at PhysicsX</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4851193101</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>75</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Simulation, Simulation Engineer, Design</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L20" t="b">
+        <v>1</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>PhysicsX</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Job Application for Research Scientist at PhysicsX</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4652633101</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>75</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Simulation, Simulation Engineer, Design</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L21" t="b">
+        <v>1</v>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>PhysicsX</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Job Application for Machine Learning Software Engineer, Research at PhysicsX</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4652630101</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>75</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Simulation, Simulation Engineer, Design</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L22" t="b">
+        <v>1</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>PhysicsX</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Job Application for Staff Machine Learning Software Engineer, Research at PhysicsX</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4851342101</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>75</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Simulation, Simulation Engineer, Design</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L23" t="b">
+        <v>1</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>PhysicsX</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Job Application for Core Services - Software Engineer (Frontend) at PhysicsX</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4824923101</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>50</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Simulation, Simulation Engineer, Design</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L24" t="b">
+        <v>1</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>PhysicsX</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Job Application for Machine Learning Engineer at PhysicsX</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4849382101</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>50</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Simulation, Simulation Engineer, Design</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L25" t="b">
+        <v>1</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>PhysicsX</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Job Application for Machine Learning Engineer at PhysicsX</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4880947101</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>50</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Simulation, Simulation Engineer, Design</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L26" t="b">
+        <v>1</v>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>PhysicsX</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Job Application for Senior Software Engineer - AI Workbench at PhysicsX</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4789290101</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>50</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Simulation, Simulation Engineer, Design</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L27" t="b">
+        <v>1</v>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>PhysicsX</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Job Application for Senior Product Designer, Client-Facing at PhysicsX</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4699630101</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>50</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Simulation, Simulation Engineer, Design</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L28" t="b">
+        <v>1</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>PhysicsX</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Job Application for Data Scientist at PhysicsX</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4880922101</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>50</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Simulation, Simulation Engineer, Design</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L29" t="b">
+        <v>1</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>PhysicsX</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Job Application for Data Scientist at PhysicsX</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4880929101</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>50</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Simulation, Simulation Engineer, Design</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L30" t="b">
+        <v>1</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>PhysicsX</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Job Application for Software Engineer - Go &amp; Python (Core Services) at PhysicsX</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/physicsx/jobs/4820418101</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>50</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Simulation, Simulation Engineer, Design</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L31" t="b">
+        <v>1</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Rheinmetal</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Operativer Einkäufer / Materialmanager (m/w/d) | Rheinmetall</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://www.rheinmetall.com/en/job/operativer_einkaeufer___materialmanager__m_w_d_/769019</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>45</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Entwicklung</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Germany, UK</t>
+        </is>
+      </c>
+      <c r="L32" t="b">
+        <v>1</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Siemens</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Early career programs in the energy sector</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://www.siemens-energy.com/global/en/home/careers/early-career-programs.html</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>41</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Germany, Netherland, Austria, UK, France, Italy, Australia</t>
+        </is>
+      </c>
+      <c r="L33" t="b">
+        <v>1</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Rheinmetal</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Angebotsleiter / Bid Manager (m/w/d) | Rheinmetall</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://www.rheinmetall.com/en/job/angebotsleiter___bid_manager__m_w_d_/766025</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>40</v>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Entwicklung, Design</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="L12" t="b">
-        <v>1</v>
-      </c>
-      <c r="M12" t="inlineStr">
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Entwicklung</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="L34" t="b">
+        <v>1</v>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Rheinmetal</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Bid &amp; Proposal Manager - Service (m/w/d) | Rheinmetall</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://www.rheinmetall.com/en/job/bid___proposal_manager_service__m_w_d_/776369</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>40</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Entwicklung</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="L35" t="b">
+        <v>1</v>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Rheinmetal</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Systemingenieur Systemanalyse und Systementwurf (m/w/d) | Rheinmetall</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>https://www.rheinmetall.com/en/job/systemingenieur_systemanalyse_und_systementwurf__m_w_d_/769955</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>40</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Entwicklung</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="L36" t="b">
+        <v>1</v>
+      </c>
+      <c r="M36" t="inlineStr">
         <is>
           <t>Matched</t>
         </is>

</xml_diff>

<commit_message>
Run: Updated Rohin job outputs 2026-06-04 21:53:26
</commit_message>
<xml_diff>
--- a/users/Rohin/outputs/JobMatches.xlsx
+++ b/users/Rohin/outputs/JobMatches.xlsx
@@ -13,6 +13,7 @@
     <sheet name="20260604_161235" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="20260604_195333" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="20260604_201725" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="20260604_215304" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -4651,15 +4652,212 @@
           <t>2026-06-04</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Rheinmetal</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Senior Expert Network &amp; Security Architecture (m/w/d) | Rheinmetall</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://www.rheinmetall.com/en/job/senior_expert_network___security_architecture__m_w_d_/778061</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>50</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Entwicklung, Design</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Germany, UK</t>
+        </is>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Rheinmetal</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Mitarbeiter Qualitätssicherung mit Schwerpunkt Mechanik (m/w/d) | Rheinmetall</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://www.rheinmetall.com/en/job/mitarbeiter_qualitaetssicherung_mit_schwerpunkt_mechanik__m_w_d_/782153</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>40</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Entwicklung</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>CrawlDate</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>PostedDate</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Keywords</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Locations</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Rheinmetal</t>
+          <t>Dawn aero</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -4669,90 +4867,31 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Senior Expert Network &amp; Security Architecture (m/w/d) | Rheinmetall</t>
+          <t>Job Application for Mechanical Engineer at Dawn Aerospace</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rheinmetall.com/en/job/senior_expert_network___security_architecture__m_w_d_/778061</t>
+          <t>https://job-boards.anz.greenhouse.io/dawnaerospace/jobs/4003811201</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Entwicklung, Design</t>
+          <t>CFD, Simulation, Fluid, Design</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Germany, UK</t>
+          <t>Netherland, France</t>
         </is>
       </c>
       <c r="L2" t="b">
         <v>1</v>
       </c>
       <c r="M2" t="inlineStr">
-        <is>
-          <t>Matched</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Rheinmetal</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Job</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Mitarbeiter Qualitätssicherung mit Schwerpunkt Mechanik (m/w/d) | Rheinmetall</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>https://www.rheinmetall.com/en/job/mitarbeiter_qualitaetssicherung_mit_schwerpunkt_mechanik__m_w_d_/782153</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
-        <v>40</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Entwicklung</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="L3" t="b">
-        <v>1</v>
-      </c>
-      <c r="M3" t="inlineStr">
         <is>
           <t>Matched</t>
         </is>

</xml_diff>

<commit_message>
Run: Updated Rohin job outputs 2026-06-05 11:26:38
</commit_message>
<xml_diff>
--- a/users/Rohin/outputs/JobMatches.xlsx
+++ b/users/Rohin/outputs/JobMatches.xlsx
@@ -14,6 +14,7 @@
     <sheet name="20260604_195333" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="20260604_201725" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="20260604_215304" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="20260605_112604" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -4849,15 +4850,154 @@
           <t>2026-06-04</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Dawn aero</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Job Application for Mechanical Engineer at Dawn Aerospace</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://job-boards.anz.greenhouse.io/dawnaerospace/jobs/4003811201</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>111</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>CFD, Simulation, Fluid, Design</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Netherland, France</t>
+        </is>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>CrawlDate</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>PostedDate</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Keywords</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Locations</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Dawn aero</t>
+          <t>Fraunhofer</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -4867,31 +5007,267 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Job Application for Mechanical Engineer at Dawn Aerospace</t>
+          <t>Wissenschaftler*in im Bereich Faserlaser Stellendetails | Fraunhofer-Gesellschaft</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://job-boards.anz.greenhouse.io/dawnaerospace/jobs/4003811201</t>
+          <t>https://jobs.fraunhofer.de/job/Ettlingen-Wissenschaftlerin-im-Bereich-Faserlaser-76275/1372052133/</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>111</v>
+        <v>85</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>CFD, Simulation, Fluid, Design</t>
+          <t>Entwicklung, Simulation, Design</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Netherland, France</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="L2" t="b">
         <v>1</v>
       </c>
       <c r="M2" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Fraunhofer</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Masterarbeit »Prozessentwicklung für SynFuels: Katalysator-Tests zur Alkoholkondensation« Stellendetails | Fraunhofer-Gesellschaft</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://jobs.fraunhofer.de/job/Oberhausen-Masterarbeit-%C2%BBProzessentwicklung-f%C3%BCr-SynFuels-Katalysator-Tests-zur-Alkoholkondensation%C2%AB-46047/1381539033/</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>80</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Fraunhofer</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Wissenschaftliche*r Mitarbeiter*in für photonisch integrierte Sensorsysteme Stellendetails | Fraunhofer-Gesellschaft</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://jobs.fraunhofer.de/job/Chemnitz-Wissenschaftlicher-Mitarbeiterin-f%C3%BCr-photonisch-integrierte-Sensorsysteme-09126/1381674133/</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>80</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Rheinmetal</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>SAP Q-Modul Key-User (m/w/d) | Rheinmetall</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://www.rheinmetall.com/en/job/sap_q_modul_key_user__m_w_d_/771131</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>40</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Entwicklung</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Fraunhofer</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Bachelor-/ Masterarbeit: »Fertigung innovativer Stackkomponenten für die PEM-Elektrolyse« Stellendetails | Fraunhofer-Gesellschaft</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://jobs.fraunhofer.de/job/Aachen-Bachelor-Masterarbeit-%C2%BBFertigung-innovativer-Stackkomponenten-f%C3%BCr-die-PEM-Elektrolyse%C2%AB-52074/1381636033/</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>40</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Entwicklung, Design</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+      <c r="M6" t="inlineStr">
         <is>
           <t>Matched</t>
         </is>

</xml_diff>

<commit_message>
Run: Updated Rohin job outputs 2026-06-08 18:58:10
</commit_message>
<xml_diff>
--- a/users/Rohin/outputs/JobMatches.xlsx
+++ b/users/Rohin/outputs/JobMatches.xlsx
@@ -15,6 +15,7 @@
     <sheet name="20260604_201725" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="20260604_215304" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="20260605_112604" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="20260608_185746" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1023,6 +1024,1164 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>CrawlDate</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>PostedDate</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Keywords</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Locations</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/java-full-stack-developer.html</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>210</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>CFD, Computational Fluid Dynamics, Simulation, Fluid, ANSYS, Design</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/junior-hpc-engineer.html</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>115</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>CFD, Simulation, ANSYS, Design</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/vertriebsassistent-sales-administrator.html</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>105</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>CFD, Simulation, Design</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/net-full-stack-developer-middle.html</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>105</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>CFD, Simulation, Design</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>EP Mannheim</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Software Engineer C++ Simulation/Distributed Systems (m/w/d)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://www.ep-group.de/job/MA1382415</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Aconext</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Career | Aconext</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://aconext.de/en/jobs?job-category=berufserfahren&amp;job-employment-type=default&amp;job-industry=default</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>95</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation, Design</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Germany, UK</t>
+        </is>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Aconext</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Career | Aconext</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://aconext.de/en/jobs/</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>95</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation, Design</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Germany, UK</t>
+        </is>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Fraunhofer</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Wissenschaftlicher Mitarbeiter (all genders) - Systemorientierte Hochfrequenz-Schaltungen Stellendetails | Fraunhofer-Gesellschaft</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://jobs.fraunhofer.de/job/Freiburg-Wissenschaftlicher-Mitarbeiter-%28all-genders%29-Systemorientierte-Hochfrequenz-Schaltungen-79108/1401915933/</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>85</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation, Design</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Fraunhofer</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Wissenschaftliche*r Mitarbeiter*in im Bereich Geothermie und Hydrogeologie Stellendetails | Fraunhofer-Gesellschaft</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://jobs.fraunhofer.de/job/Bochum-Wissenschaftlicher-Mitarbeiterin-im-Bereich-Geothermie-und-Hydrogeologie-44801/1401873333/</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>80</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L10" t="b">
+        <v>1</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/senior-sales-manager-ict-e-system-integration.html</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>65</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Simulation, ANSYS, Design</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="b">
+        <v>1</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/mechanical-application-engineer.html</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>65</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Simulation, ANSYS, Design</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="b">
+        <v>1</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/vertriebsbeauftragter-simulationslosungen.html</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>65</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Simulation, ANSYS, Design</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="b">
+        <v>1</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/sistemista-it-infrastructure-operations-specialist.html</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>65</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Simulation, ANSYS, Design</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="b">
+        <v>1</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/career.html</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>65</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Simulation, ANSYS, Design</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="b">
+        <v>1</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>65</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Simulation, ANSYS, Design</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="b">
+        <v>1</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/tecnico-sistemista-hpc.html</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>60</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Simulation, Design</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="L17" t="b">
+        <v>1</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Rheinmetal</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Technischer Prüfer F-35 (m/w/d) | Rheinmetall</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://www.rheinmetall.com/en/job/technischer_pruefer_f_35__m_w_d_/772148</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>45</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Entwicklung</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Germany, UK</t>
+        </is>
+      </c>
+      <c r="L18" t="b">
+        <v>1</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>EP Mannheim</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Softwareentwickler .NET / Backend Developer (m/w/d)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://www.ep-group.de/job/BE1382409</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>40</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Entwicklung, Design</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L19" t="b">
+        <v>1</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Fraunhofer</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Bachelorand / Masterand - Evaluation von Verpackungskonzepten für Fresh-Cut-Salate (all genders) Stellendetails | Fraunhofer-Gesellschaft</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://jobs.fraunhofer.de/job/Freising-Bachelorand-Masterand-Evaluation-von-Verpackungskonzepten-f%C3%BCr-Fresh-Cut-Salate-%28all-genders%29-85354/1373549433/</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>40</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Entwicklung, Design</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L20" t="b">
+        <v>1</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -4989,7 +6148,6 @@
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>Fraunhofer</t>
@@ -5048,7 +6206,6 @@
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>Fraunhofer</t>
@@ -5107,7 +6264,6 @@
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>Fraunhofer</t>
@@ -5166,7 +6322,6 @@
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>Rheinmetal</t>
@@ -5225,7 +6380,6 @@
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>Fraunhofer</t>

</xml_diff>

<commit_message>
Run: Updated Rohin job outputs 2026-06-09 18:12:26
</commit_message>
<xml_diff>
--- a/users/Rohin/outputs/JobMatches.xlsx
+++ b/users/Rohin/outputs/JobMatches.xlsx
@@ -16,6 +16,7 @@
     <sheet name="20260604_215304" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="20260605_112604" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="20260608_185746" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="20260609_181149" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1111,15 +1112,1143 @@
           <t>2026-06-08</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/java-full-stack-developer.html</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>210</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>CFD, Computational Fluid Dynamics, Simulation, Fluid, ANSYS, Design</t>
+        </is>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/junior-hpc-engineer.html</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>115</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>CFD, Simulation, ANSYS, Design</t>
+        </is>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/vertriebsassistent-sales-administrator.html</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>105</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>CFD, Simulation, Design</t>
+        </is>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/net-full-stack-developer-middle.html</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>105</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>CFD, Simulation, Design</t>
+        </is>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>EP Mannheim</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Software Engineer C++ Simulation/Distributed Systems (m/w/d)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://www.ep-group.de/job/MA1382415</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation</t>
+        </is>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Aconext</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Career | Aconext</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://aconext.de/en/jobs?job-category=berufserfahren&amp;job-employment-type=default&amp;job-industry=default</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>95</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation, Design</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Germany, UK</t>
+        </is>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Aconext</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Career | Aconext</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://aconext.de/en/jobs/</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>95</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation, Design</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Germany, UK</t>
+        </is>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Fraunhofer</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Wissenschaftlicher Mitarbeiter (all genders) - Systemorientierte Hochfrequenz-Schaltungen Stellendetails | Fraunhofer-Gesellschaft</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://jobs.fraunhofer.de/job/Freiburg-Wissenschaftlicher-Mitarbeiter-%28all-genders%29-Systemorientierte-Hochfrequenz-Schaltungen-79108/1401915933/</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>85</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation, Design</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Fraunhofer</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Wissenschaftliche*r Mitarbeiter*in im Bereich Geothermie und Hydrogeologie Stellendetails | Fraunhofer-Gesellschaft</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://jobs.fraunhofer.de/job/Bochum-Wissenschaftlicher-Mitarbeiterin-im-Bereich-Geothermie-und-Hydrogeologie-44801/1401873333/</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>80</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L10" t="b">
+        <v>1</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/senior-sales-manager-ict-e-system-integration.html</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>65</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Simulation, ANSYS, Design</t>
+        </is>
+      </c>
+      <c r="L11" t="b">
+        <v>1</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/mechanical-application-engineer.html</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>65</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Simulation, ANSYS, Design</t>
+        </is>
+      </c>
+      <c r="L12" t="b">
+        <v>1</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/vertriebsbeauftragter-simulationslosungen.html</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>65</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Simulation, ANSYS, Design</t>
+        </is>
+      </c>
+      <c r="L13" t="b">
+        <v>1</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/sistemista-it-infrastructure-operations-specialist.html</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>65</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Simulation, ANSYS, Design</t>
+        </is>
+      </c>
+      <c r="L14" t="b">
+        <v>1</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/career.html</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>65</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Simulation, ANSYS, Design</t>
+        </is>
+      </c>
+      <c r="L15" t="b">
+        <v>1</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>65</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Simulation, ANSYS, Design</t>
+        </is>
+      </c>
+      <c r="L16" t="b">
+        <v>1</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Enginsoft</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.enginsoft.com/careers/careers/tecnico-sistemista-hpc.html</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>60</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Simulation, Design</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="L17" t="b">
+        <v>1</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Rheinmetal</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Technischer Prüfer F-35 (m/w/d) | Rheinmetall</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://www.rheinmetall.com/en/job/technischer_pruefer_f_35__m_w_d_/772148</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>45</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Entwicklung</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Germany, UK</t>
+        </is>
+      </c>
+      <c r="L18" t="b">
+        <v>1</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>EP Mannheim</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Softwareentwickler .NET / Backend Developer (m/w/d)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://www.ep-group.de/job/BE1382409</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>40</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Entwicklung, Design</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L19" t="b">
+        <v>1</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Fraunhofer</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Bachelorand / Masterand - Evaluation von Verpackungskonzepten für Fresh-Cut-Salate (all genders) Stellendetails | Fraunhofer-Gesellschaft</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://jobs.fraunhofer.de/job/Freising-Bachelorand-Masterand-Evaluation-von-Verpackungskonzepten-f%C3%BCr-Fresh-Cut-Salate-%28all-genders%29-85354/1373549433/</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>40</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Entwicklung, Design</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L20" t="b">
+        <v>1</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>CrawlDate</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>PostedDate</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Keywords</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Locations</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Enginsoft</t>
+          <t>University of Siegen</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1129,23 +2258,27 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+          <t>Akademische Rätin / Akademischer Rat aZ - Lehrstuhl für Produktentwicklung Stellendetails | Universität Siegen</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.enginsoft.com/careers/careers/java-full-stack-developer.html</t>
+          <t>https://jobs.uni-siegen.de/job/Akademische-R%C3%A4tin-Akademischer-Rat-aZ-Lehrstuhl-f%C3%BCr-Produktentwicklung-57076/1399826033/</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>210</v>
+        <v>85</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>CFD, Computational Fluid Dynamics, Simulation, Fluid, ANSYS, Design</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr"/>
+          <t>Entwicklung, Simulation, Design</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
       <c r="L2" t="b">
         <v>1</v>
       </c>
@@ -1158,23 +2291,23 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Enginsoft</t>
+          <t>University of Siegen</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1184,23 +2317,27 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+          <t>Wissenschaftliche/r Mitarbeiter/in - Lehrstuhl für Tragkonstruktion Stellendetails | Universität Siegen</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.enginsoft.com/careers/careers/junior-hpc-engineer.html</t>
+          <t>https://jobs.uni-siegen.de/job/Wissenschaftlicher-Mitarbeiterin-Lehrstuhl-f%C3%BCr-Tragkonstruktion-57076/1388638133/</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>CFD, Simulation, ANSYS, Design</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr"/>
+          <t>Entwicklung, Simulation</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
       <c r="L3" t="b">
         <v>1</v>
       </c>
@@ -1213,23 +2350,23 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Enginsoft</t>
+          <t>Fraunhofer</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1239,23 +2376,27 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+          <t>BACK-END-ENTWICKLER*IN (all genders) Stellendetails | Fraunhofer-Gesellschaft</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.enginsoft.com/careers/careers/vertriebsassistent-sales-administrator.html</t>
+          <t>https://jobs.fraunhofer.de/job/Kaiserslautern-BACK-END-ENTWICKLERIN-%28all-genders%29-67663/1392421633/</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>CFD, Simulation, Design</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr"/>
+          <t>Entwicklung, Simulation</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
       <c r="L4" t="b">
         <v>1</v>
       </c>
@@ -1268,23 +2409,23 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Enginsoft</t>
+          <t>University of Siegen</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1294,23 +2435,27 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+          <t>Mitarbeiter/in - ZIMT - IT-System Engineer im Bereich KI-Anwendungen und High Performance Computing Stellendetails | Universität Siegen</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.enginsoft.com/careers/careers/net-full-stack-developer-middle.html</t>
+          <t>https://jobs.uni-siegen.de/job/Mitarbeiterin-ZIMT-IT-System-Engineer-im-Bereich-KI-Anwendungen-und-High-Performance-Computing-57076/1401238033/</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>CFD, Simulation, Design</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr"/>
+          <t>Entwicklung, Simulation</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
       <c r="L5" t="b">
         <v>1</v>
       </c>
@@ -1323,18 +2468,18 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>EP Mannheim</t>
+          <t>Rheinmetal</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1349,23 +2494,27 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Software Engineer C++ Simulation/Distributed Systems (m/w/d)</t>
+          <t>Configuration / Production Data Analyst F-35 (m/w/d) | Rheinmetall</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.ep-group.de/job/MA1382415</t>
+          <t>https://www.rheinmetall.com/en/job/configuration___production_data_analyst_f_35__m_w_d_/1060088</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Entwicklung, Simulation</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr"/>
+          <t>Entwicklung, Design</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Germany, UK</t>
+        </is>
+      </c>
       <c r="L6" t="b">
         <v>1</v>
       </c>
@@ -1378,18 +2527,18 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Aconext</t>
+          <t>Rheinmetal</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1404,20 +2553,20 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Career | Aconext</t>
+          <t>Change and Configuration Manager F-35 (m/w/d) | Rheinmetall</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://aconext.de/en/jobs?job-category=berufserfahren&amp;job-employment-type=default&amp;job-industry=default</t>
+          <t>https://www.rheinmetall.com/en/job/change_and_configuration_manager_f_35__m_w_d_/1060103</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Entwicklung, Simulation, Design</t>
+          <t>Entwicklung</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1437,18 +2586,18 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Aconext</t>
+          <t>Rheinmetal</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1463,20 +2612,20 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Career | Aconext</t>
+          <t>Infrastrukturkoordinator (m/w/d) | Rheinmetall</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://aconext.de/en/jobs/</t>
+          <t>https://www.rheinmetall.com/en/job/infrastrukturkoordinator__m_w_d_/1060118</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Entwicklung, Simulation, Design</t>
+          <t>Entwicklung</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1496,18 +2645,18 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Fraunhofer</t>
+          <t>Grob Aircraft</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1522,20 +2671,20 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Wissenschaftlicher Mitarbeiter (all genders) - Systemorientierte Hochfrequenz-Schaltungen Stellendetails | Fraunhofer-Gesellschaft</t>
+          <t>Offene Stellen - Grob Aircraft SE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://jobs.fraunhofer.de/job/Freiburg-Wissenschaftlicher-Mitarbeiter-%28all-genders%29-Systemorientierte-Hochfrequenz-Schaltungen-79108/1401915933/</t>
+          <t>https://jobs.grob-aircraft.com/jobs/show_more?page=2</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>85</v>
+        <v>40</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Entwicklung, Simulation, Design</t>
+          <t>Entwicklung, Design</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1555,12 +2704,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -1581,20 +2730,20 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Wissenschaftliche*r Mitarbeiter*in im Bereich Geothermie und Hydrogeologie Stellendetails | Fraunhofer-Gesellschaft</t>
+          <t>Master- oder Bachelorarbeit: Additive Fertigung (LB‑PBF) &amp; Mikrostrukturanalyse Stellendetails | Fraunhofer-Gesellschaft</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://jobs.fraunhofer.de/job/Bochum-Wissenschaftlicher-Mitarbeiterin-im-Bereich-Geothermie-und-Hydrogeologie-44801/1401873333/</t>
+          <t>https://jobs.fraunhofer.de/job/Freiburg-Master-oder-Bachelorarbeit-Additive-Fertigung-%28LB%E2%80%91PBF%29-&amp;-Mikrostrukturanalyse-79104/1293641401/</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Entwicklung, Simulation</t>
+          <t>Entwicklung, Design</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1614,23 +2763,23 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Enginsoft</t>
+          <t>Rheinmetal</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1640,538 +2789,31 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Technology transfer and simulation software solutions | EnginSoft</t>
+          <t>Maschinen- und Anlagenführer Artilleriewerk - automatisierte Lackieranlage (m/w/d) | Rheinmetall</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.enginsoft.com/careers/careers/senior-sales-manager-ict-e-system-integration.html</t>
+          <t>https://www.rheinmetall.com/en/job/maschinen_und_anlagenfuehrer_artilleriewerk_automatisierte_lackieranlage__m_w_d_/1060100</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Simulation, ANSYS, Design</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr"/>
+          <t>Entwicklung</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
       <c r="L11" t="b">
         <v>1</v>
       </c>
       <c r="M11" t="inlineStr">
-        <is>
-          <t>Matched</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Enginsoft</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Sweden</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Job</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Technology transfer and simulation software solutions | EnginSoft</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>https://www.enginsoft.com/careers/careers/mechanical-application-engineer.html</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>65</v>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Simulation, ANSYS, Design</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="b">
-        <v>1</v>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>Matched</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Enginsoft</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Sweden</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Job</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Technology transfer and simulation software solutions | EnginSoft</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>https://www.enginsoft.com/careers/careers/vertriebsbeauftragter-simulationslosungen.html</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>65</v>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Simulation, ANSYS, Design</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="b">
-        <v>1</v>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>Matched</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Enginsoft</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Sweden</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Job</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Technology transfer and simulation software solutions | EnginSoft</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>https://www.enginsoft.com/careers/careers/sistemista-it-infrastructure-operations-specialist.html</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>65</v>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Simulation, ANSYS, Design</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="b">
-        <v>1</v>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>Matched</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Enginsoft</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Sweden</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Job</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Technology transfer and simulation software solutions | EnginSoft</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>https://www.enginsoft.com/careers/career.html</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>65</v>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Simulation, ANSYS, Design</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="b">
-        <v>1</v>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>Matched</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Enginsoft</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Sweden</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Job</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Technology transfer and simulation software solutions | EnginSoft</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>https://www.enginsoft.com/careers/careers/</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>65</v>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Simulation, ANSYS, Design</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="b">
-        <v>1</v>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>Matched</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Enginsoft</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Sweden</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Job</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Technology transfer and simulation software solutions | EnginSoft</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>https://www.enginsoft.com/careers/careers/tecnico-sistemista-hpc.html</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>60</v>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Simulation, Design</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="L17" t="b">
-        <v>1</v>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>Matched</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Rheinmetal</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Job</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Technischer Prüfer F-35 (m/w/d) | Rheinmetall</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>https://www.rheinmetall.com/en/job/technischer_pruefer_f_35__m_w_d_/772148</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>45</v>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Entwicklung</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>Germany, UK</t>
-        </is>
-      </c>
-      <c r="L18" t="b">
-        <v>1</v>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>Matched</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>EP Mannheim</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Job</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Softwareentwickler .NET / Backend Developer (m/w/d)</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>https://www.ep-group.de/job/BE1382409</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>40</v>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Entwicklung, Design</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="L19" t="b">
-        <v>1</v>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>Matched</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Fraunhofer</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Job</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Bachelorand / Masterand - Evaluation von Verpackungskonzepten für Fresh-Cut-Salate (all genders) Stellendetails | Fraunhofer-Gesellschaft</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>https://jobs.fraunhofer.de/job/Freising-Bachelorand-Masterand-Evaluation-von-Verpackungskonzepten-f%C3%BCr-Fresh-Cut-Salate-%28all-genders%29-85354/1373549433/</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>40</v>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Entwicklung, Design</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="L20" t="b">
-        <v>1</v>
-      </c>
-      <c r="M20" t="inlineStr">
         <is>
           <t>Matched</t>
         </is>

</xml_diff>

<commit_message>
Run: Updated Rohin job outputs 2026-06-11 13:02:19
</commit_message>
<xml_diff>
--- a/users/Rohin/outputs/JobMatches.xlsx
+++ b/users/Rohin/outputs/JobMatches.xlsx
@@ -17,6 +17,7 @@
     <sheet name="20260605_112604" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="20260608_185746" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="20260609_181149" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="20260611_130153" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -2240,10 +2241,671 @@
           <t>2026-06-09</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>University of Siegen</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Akademische Rätin / Akademischer Rat aZ - Lehrstuhl für Produktentwicklung Stellendetails | Universität Siegen</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://jobs.uni-siegen.de/job/Akademische-R%C3%A4tin-Akademischer-Rat-aZ-Lehrstuhl-f%C3%BCr-Produktentwicklung-57076/1399826033/</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>85</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation, Design</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>University of Siegen</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Wissenschaftliche/r Mitarbeiter/in - Lehrstuhl für Tragkonstruktion Stellendetails | Universität Siegen</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://jobs.uni-siegen.de/job/Wissenschaftlicher-Mitarbeiterin-Lehrstuhl-f%C3%BCr-Tragkonstruktion-57076/1388638133/</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>80</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Fraunhofer</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>BACK-END-ENTWICKLER*IN (all genders) Stellendetails | Fraunhofer-Gesellschaft</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://jobs.fraunhofer.de/job/Kaiserslautern-BACK-END-ENTWICKLERIN-%28all-genders%29-67663/1392421633/</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>80</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>University of Siegen</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Mitarbeiter/in - ZIMT - IT-System Engineer im Bereich KI-Anwendungen und High Performance Computing Stellendetails | Universität Siegen</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://jobs.uni-siegen.de/job/Mitarbeiterin-ZIMT-IT-System-Engineer-im-Bereich-KI-Anwendungen-und-High-Performance-Computing-57076/1401238033/</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>80</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Entwicklung, Simulation</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Rheinmetal</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Configuration / Production Data Analyst F-35 (m/w/d) | Rheinmetall</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://www.rheinmetall.com/en/job/configuration___production_data_analyst_f_35__m_w_d_/1060088</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>50</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Entwicklung, Design</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Germany, UK</t>
+        </is>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Rheinmetal</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Change and Configuration Manager F-35 (m/w/d) | Rheinmetall</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://www.rheinmetall.com/en/job/change_and_configuration_manager_f_35__m_w_d_/1060103</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>45</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Entwicklung</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Germany, UK</t>
+        </is>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Rheinmetal</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Infrastrukturkoordinator (m/w/d) | Rheinmetall</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.rheinmetall.com/en/job/infrastrukturkoordinator__m_w_d_/1060118</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>45</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Entwicklung</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Germany, UK</t>
+        </is>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Grob Aircraft</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Offene Stellen - Grob Aircraft SE</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://jobs.grob-aircraft.com/jobs/show_more?page=2</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>40</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Entwicklung, Design</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Fraunhofer</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Master- oder Bachelorarbeit: Additive Fertigung (LB‑PBF) &amp; Mikrostrukturanalyse Stellendetails | Fraunhofer-Gesellschaft</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://jobs.fraunhofer.de/job/Freiburg-Master-oder-Bachelorarbeit-Additive-Fertigung-%28LB%E2%80%91PBF%29-&amp;-Mikrostrukturanalyse-79104/1293641401/</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>40</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Entwicklung, Design</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="L10" t="b">
+        <v>1</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Rheinmetal</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Maschinen- und Anlagenführer Artilleriewerk - automatisierte Lackieranlage (m/w/d) | Rheinmetall</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://www.rheinmetall.com/en/job/maschinen_und_anlagenfuehrer_artilleriewerk_automatisierte_lackieranlage__m_w_d_/1060100</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>40</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Entwicklung</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="L11" t="b">
+        <v>1</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>CrawlDate</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>PostedDate</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Keywords</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Locations</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Matched</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>University of Siegen</t>
+          <t>Rocket Factory</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -2258,25 +2920,25 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Akademische Rätin / Akademischer Rat aZ - Lehrstuhl für Produktentwicklung Stellendetails | Universität Siegen</t>
+          <t>Job Application for Senior Development Engineer - Valves (m/f/d) at Rocket Factory Augsburg AG (EN)</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://jobs.uni-siegen.de/job/Akademische-R%C3%A4tin-Akademischer-Rat-aZ-Lehrstuhl-f%C3%BCr-Produktentwicklung-57076/1399826033/</t>
+          <t>https://job-boards.eu.greenhouse.io/rocketfactoryaugsburgag/jobs/4888885101</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Entwicklung, Simulation, Design</t>
+          <t>Fluid, Design</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Germany, UK</t>
         </is>
       </c>
       <c r="L2" t="b">
@@ -2291,18 +2953,18 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>University of Siegen</t>
+          <t>ÒKAPI</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -2317,25 +2979,25 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Wissenschaftliche/r Mitarbeiter/in - Lehrstuhl für Tragkonstruktion Stellendetails | Universität Siegen</t>
+          <t>(Junior) Backend-Entwickler (Java / Python, Microservices) (m/w/d) – Befristeter Vertrag | Jobs bei OKAPI:Orbits GmbH</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://jobs.uni-siegen.de/job/Wissenschaftlicher-Mitarbeiterin-Lehrstuhl-f%C3%BCr-Tragkonstruktion-57076/1388638133/</t>
+          <t>https://okapiorbits.jobs.personio.de/job/2666049</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Entwicklung, Simulation</t>
+          <t>Entwicklung, Design</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Germany, UK</t>
         </is>
       </c>
       <c r="L3" t="b">
@@ -2350,18 +3012,18 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Fraunhofer</t>
+          <t>ÒKAPI</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -2376,25 +3038,25 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>BACK-END-ENTWICKLER*IN (all genders) Stellendetails | Fraunhofer-Gesellschaft</t>
+          <t>(Junior) Backend-Entwickler (Java / Python, Microservices) (m/w/d) – Befristeter Vertrag | Jobs bei OKAPI:Orbits GmbH</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://jobs.fraunhofer.de/job/Kaiserslautern-BACK-END-ENTWICKLERIN-%28all-genders%29-67663/1392421633/</t>
+          <t>https://okapiorbits.jobs.personio.de/job/2407543</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Entwicklung, Simulation</t>
+          <t>Entwicklung, Design</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Germany, UK</t>
         </is>
       </c>
       <c r="L4" t="b">
@@ -2409,18 +3071,18 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>University of Siegen</t>
+          <t>Rheinmetal</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -2435,25 +3097,25 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Mitarbeiter/in - ZIMT - IT-System Engineer im Bereich KI-Anwendungen und High Performance Computing Stellendetails | Universität Siegen</t>
+          <t>Projektmanager Vertrieb (m/w/d) | Rheinmetall</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://jobs.uni-siegen.de/job/Mitarbeiterin-ZIMT-IT-System-Engineer-im-Bereich-KI-Anwendungen-und-High-Performance-Computing-57076/1401238033/</t>
+          <t>https://www.rheinmetall.com/en/job/projektmanager_vertrieb__m_w_d_/783239</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Entwicklung, Simulation</t>
+          <t>Entwicklung</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Germany, UK</t>
         </is>
       </c>
       <c r="L5" t="b">
@@ -2468,12 +3130,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -2494,20 +3156,20 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Configuration / Production Data Analyst F-35 (m/w/d) | Rheinmetall</t>
+          <t>Fertigungssteuerer (m/w/d) | Rheinmetall</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rheinmetall.com/en/job/configuration___production_data_analyst_f_35__m_w_d_/1060088</t>
+          <t>https://www.rheinmetall.com/en/job/fertigungssteuerer__m_w_d_/783200</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Entwicklung, Design</t>
+          <t>Entwicklung</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -2519,301 +3181,6 @@
         <v>1</v>
       </c>
       <c r="M6" t="inlineStr">
-        <is>
-          <t>Matched</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Rheinmetal</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Job</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Change and Configuration Manager F-35 (m/w/d) | Rheinmetall</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>https://www.rheinmetall.com/en/job/change_and_configuration_manager_f_35__m_w_d_/1060103</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>45</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Entwicklung</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Germany, UK</t>
-        </is>
-      </c>
-      <c r="L7" t="b">
-        <v>1</v>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>Matched</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Rheinmetal</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Job</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Infrastrukturkoordinator (m/w/d) | Rheinmetall</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>https://www.rheinmetall.com/en/job/infrastrukturkoordinator__m_w_d_/1060118</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>45</v>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Entwicklung</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Germany, UK</t>
-        </is>
-      </c>
-      <c r="L8" t="b">
-        <v>1</v>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>Matched</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Grob Aircraft</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Job</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Offene Stellen - Grob Aircraft SE</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>https://jobs.grob-aircraft.com/jobs/show_more?page=2</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>40</v>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Entwicklung, Design</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="L9" t="b">
-        <v>1</v>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>Matched</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Fraunhofer</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Job</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Master- oder Bachelorarbeit: Additive Fertigung (LB‑PBF) &amp; Mikrostrukturanalyse Stellendetails | Fraunhofer-Gesellschaft</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>https://jobs.fraunhofer.de/job/Freiburg-Master-oder-Bachelorarbeit-Additive-Fertigung-%28LB%E2%80%91PBF%29-&amp;-Mikrostrukturanalyse-79104/1293641401/</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>40</v>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Entwicklung, Design</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="L10" t="b">
-        <v>1</v>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>Matched</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Rheinmetal</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Job</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Maschinen- und Anlagenführer Artilleriewerk - automatisierte Lackieranlage (m/w/d) | Rheinmetall</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>https://www.rheinmetall.com/en/job/maschinen_und_anlagenfuehrer_artilleriewerk_automatisierte_lackieranlage__m_w_d_/1060100</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>40</v>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Entwicklung</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="L11" t="b">
-        <v>1</v>
-      </c>
-      <c r="M11" t="inlineStr">
         <is>
           <t>Matched</t>
         </is>

</xml_diff>